<commit_message>
updated the Excel file
</commit_message>
<xml_diff>
--- a/component_end_dates.xlsx
+++ b/component_end_dates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\97250\Documents\CoreStorm_git\CoreStorm_RV32I\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB5C0651-0745-484B-ABFF-CE6D0C6FEA36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5A3E642-E238-46AB-A114-9578D730E985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{58139526-2888-40EA-BA21-B55B9EAF3B56}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="68">
   <si>
     <t>Task_moudel</t>
   </si>
@@ -980,7 +980,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="14.25">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="8" t="s">
         <v>4</v>
       </c>
       <c r="B22" t="s">
@@ -988,6 +988,9 @@
       </c>
       <c r="D22" t="s">
         <v>44</v>
+      </c>
+      <c r="E22" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="14.25">

</xml_diff>

<commit_message>
adding modules and test benches
</commit_message>
<xml_diff>
--- a/component_end_dates.xlsx
+++ b/component_end_dates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\97250\Documents\CoreStorm_git\CoreStorm_RV32I\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE5C5DA-FED1-4F30-8F6A-79139C115554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88F40C13-3569-4B41-A98E-9397D4FCD0CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{58139526-2888-40EA-BA21-B55B9EAF3B56}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="71">
   <si>
     <t>Task_moudel</t>
   </si>
@@ -246,13 +246,16 @@
   </si>
   <si>
     <t>tcm_mem_ram</t>
+  </si>
+  <si>
+    <t>dport_axi_fifo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -290,6 +293,12 @@
       <color rgb="FFFF0000"/>
       <name val="Arial Unicode MS"/>
       <charset val="177"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="5">
@@ -330,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -340,6 +349,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -674,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9373D2A7-8D80-423E-9070-95B67CA8F36B}">
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.375" style="1" customWidth="1"/>
@@ -842,7 +853,7 @@
       </c>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="7" t="s">
         <v>55</v>
       </c>
       <c r="B10" t="s">
@@ -850,6 +861,9 @@
       </c>
       <c r="D10" t="s">
         <v>40</v>
+      </c>
+      <c r="E10" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -868,7 +882,7 @@
       <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="7" t="s">
         <v>57</v>
       </c>
       <c r="B12" t="s">
@@ -877,10 +891,13 @@
       <c r="D12" t="s">
         <v>38</v>
       </c>
+      <c r="E12" t="s">
+        <v>48</v>
+      </c>
       <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="7" t="s">
         <v>58</v>
       </c>
       <c r="B13" t="s">
@@ -888,6 +905,9 @@
       </c>
       <c r="D13" t="s">
         <v>39</v>
+      </c>
+      <c r="E13" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -945,14 +965,17 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="7" t="s">
         <v>63</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D18" t="s">
         <v>42</v>
+      </c>
+      <c r="E18" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -964,14 +987,17 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="7" t="s">
         <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D20" t="s">
         <v>44</v>
+      </c>
+      <c r="E20" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1094,36 +1120,42 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="14.25">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="8" t="s">
         <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D31" t="s">
         <v>45</v>
       </c>
+      <c r="E31" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="32" spans="1:5" ht="14.25">
-      <c r="A32" s="2" t="s">
-        <v>13</v>
+      <c r="A32" s="8" t="s">
+        <v>70</v>
       </c>
       <c r="B32" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D32" t="s">
         <v>45</v>
       </c>
+      <c r="E32" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="33" spans="1:5" ht="14.25">
       <c r="A33" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B33" t="s">
         <v>24</v>
       </c>
       <c r="D33" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E33" t="s">
         <v>48</v>
@@ -1131,7 +1163,7 @@
     </row>
     <row r="34" spans="1:5" ht="14.25">
       <c r="A34" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B34" t="s">
         <v>24</v>
@@ -1145,7 +1177,7 @@
     </row>
     <row r="35" spans="1:5" ht="14.25">
       <c r="A35" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B35" t="s">
         <v>24</v>
@@ -1158,19 +1190,22 @@
       </c>
     </row>
     <row r="36" spans="1:5" ht="14.25">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B36" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" t="s">
+        <v>47</v>
+      </c>
+      <c r="E36" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="14.25">
+      <c r="A37" s="10" t="s">
         <v>17</v>
-      </c>
-      <c r="B36" t="s">
-        <v>27</v>
-      </c>
-      <c r="D36" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="14.25">
-      <c r="A37" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="B37" t="s">
         <v>24</v>
@@ -1178,32 +1213,35 @@
       <c r="D37" t="s">
         <v>46</v>
       </c>
+      <c r="E37" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="38" spans="1:5" ht="14.25">
-      <c r="A38" s="5" t="s">
-        <v>19</v>
+      <c r="A38" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="B38" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D38" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="14.25">
-      <c r="A39" s="2" t="s">
-        <v>20</v>
+      <c r="A39" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="B39" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D39" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="14.25">
-      <c r="A40" s="2" t="s">
-        <v>21</v>
+      <c r="A40" s="8" t="s">
+        <v>20</v>
       </c>
       <c r="B40" t="s">
         <v>24</v>
@@ -1211,10 +1249,13 @@
       <c r="D40" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="41" spans="1:5">
-      <c r="A41" s="7" t="s">
-        <v>69</v>
+      <c r="E40" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="14.25">
+      <c r="A41" s="8" t="s">
+        <v>21</v>
       </c>
       <c r="B41" t="s">
         <v>24</v>
@@ -1223,6 +1264,20 @@
         <v>46</v>
       </c>
       <c r="E41" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="14.25">
+      <c r="A42" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B42" t="s">
+        <v>24</v>
+      </c>
+      <c r="D42" t="s">
+        <v>46</v>
+      </c>
+      <c r="E42" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adding the top module
</commit_message>
<xml_diff>
--- a/component_end_dates.xlsx
+++ b/component_end_dates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\97250\Documents\CoreStorm_git\CoreStorm_RV32I\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE6CFD5-B8F7-4F07-8F85-42758084743F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D871EB5-10E3-4CF5-8990-6F7AE58541FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{58139526-2888-40EA-BA21-B55B9EAF3B56}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="72">
   <si>
     <t>Task_moudel</t>
   </si>
@@ -258,7 +258,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -289,13 +289,6 @@
       <family val="2"/>
       <charset val="177"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial Unicode MS"/>
-      <charset val="177"/>
     </font>
     <font>
       <b/>
@@ -347,18 +340,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -721,7 +713,7 @@
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B2" t="s">
@@ -744,7 +736,7 @@
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B3" t="s">
@@ -764,7 +756,7 @@
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>50</v>
       </c>
       <c r="B4" t="s">
@@ -784,7 +776,7 @@
       </c>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>51</v>
       </c>
       <c r="B5" t="s">
@@ -799,13 +791,13 @@
       <c r="E5" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="6"/>
+      <c r="F5" s="5"/>
       <c r="I5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>52</v>
       </c>
       <c r="B6" t="s">
@@ -819,7 +811,7 @@
       </c>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>53</v>
       </c>
       <c r="B7" t="s">
@@ -833,7 +825,7 @@
       </c>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>65</v>
       </c>
       <c r="B8" t="s">
@@ -847,7 +839,7 @@
       </c>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>66</v>
       </c>
       <c r="B9" t="s">
@@ -861,7 +853,7 @@
       </c>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B10" t="s">
@@ -875,7 +867,7 @@
       </c>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="6" t="s">
         <v>55</v>
       </c>
       <c r="B11" t="s">
@@ -887,10 +879,10 @@
       <c r="E11" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="6"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>56</v>
       </c>
       <c r="B12" t="s">
@@ -902,10 +894,10 @@
       <c r="E12" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="6"/>
+      <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>57</v>
       </c>
       <c r="B13" t="s">
@@ -919,7 +911,7 @@
       </c>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>58</v>
       </c>
       <c r="B14" t="s">
@@ -933,7 +925,7 @@
       </c>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="6" t="s">
         <v>59</v>
       </c>
       <c r="B15" t="s">
@@ -956,10 +948,10 @@
       <c r="D16" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="5"/>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>61</v>
       </c>
       <c r="B17" t="s">
@@ -973,7 +965,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>62</v>
       </c>
       <c r="B18" t="s">
@@ -995,7 +987,7 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="6" t="s">
         <v>64</v>
       </c>
       <c r="B20" t="s">
@@ -1020,7 +1012,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="14.25">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="7" t="s">
         <v>4</v>
       </c>
       <c r="B22" t="s">
@@ -1034,7 +1026,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="14.25">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="7" t="s">
         <v>67</v>
       </c>
       <c r="B23" t="s">
@@ -1048,7 +1040,7 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="14.25">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B24" t="s">
@@ -1128,7 +1120,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="14.25">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B31" t="s">
@@ -1142,7 +1134,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="14.25">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="7" t="s">
         <v>69</v>
       </c>
       <c r="B32" t="s">
@@ -1156,7 +1148,7 @@
       </c>
     </row>
     <row r="33" spans="1:5" ht="14.25">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B33" t="s">
@@ -1170,7 +1162,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" ht="14.25">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B34" t="s">
@@ -1184,7 +1176,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" ht="14.25">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="7" t="s">
         <v>15</v>
       </c>
       <c r="B35" t="s">
@@ -1198,7 +1190,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" ht="14.25">
-      <c r="A36" s="8" t="s">
+      <c r="A36" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B36" t="s">
@@ -1212,7 +1204,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" ht="14.25">
-      <c r="A37" s="10" t="s">
+      <c r="A37" s="9" t="s">
         <v>17</v>
       </c>
       <c r="B37" t="s">
@@ -1226,7 +1218,7 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="14.25">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="7" t="s">
         <v>70</v>
       </c>
       <c r="B38" t="s">
@@ -1235,20 +1227,26 @@
       <c r="D38" t="s">
         <v>45</v>
       </c>
+      <c r="E38" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="39" spans="1:5" ht="14.25">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="9" t="s">
         <v>18</v>
       </c>
       <c r="B39" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D39" t="s">
         <v>45</v>
       </c>
+      <c r="E39" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="40" spans="1:5" ht="14.25">
-      <c r="A40" s="8" t="s">
+      <c r="A40" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B40" t="s">
@@ -1262,7 +1260,7 @@
       </c>
     </row>
     <row r="41" spans="1:5" ht="14.25">
-      <c r="A41" s="8" t="s">
+      <c r="A41" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B41" t="s">
@@ -1276,7 +1274,7 @@
       </c>
     </row>
     <row r="42" spans="1:5" ht="14.25">
-      <c r="A42" s="9" t="s">
+      <c r="A42" s="8" t="s">
         <v>68</v>
       </c>
       <c r="B42" t="s">
@@ -1290,7 +1288,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="14.25">
-      <c r="A43" s="9" t="s">
+      <c r="A43" s="8" t="s">
         <v>71</v>
       </c>
       <c r="B43" t="s">

</xml_diff>